<commit_message>
Hice una primera iteracion del main completa con mi dataset de prueba de Inglaterra. Al menos da algo. Queda revisar desde construct_data hasta modelling.
</commit_message>
<xml_diff>
--- a/p3_data_preparation/data/England/df_integrated.xlsx
+++ b/p3_data_preparation/data/England/df_integrated.xlsx
@@ -941,16 +941,16 @@
         <v>5</v>
       </c>
       <c r="BG2" t="n">
-        <v>24.22222222222222</v>
+        <v>24.77777777777778</v>
       </c>
       <c r="BH2" t="n">
-        <v>177.6666666666667</v>
+        <v>178.7777777777778</v>
       </c>
       <c r="BI2" t="n">
-        <v>76.77777777777777</v>
+        <v>77</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.5002158237542789</v>
+        <v>0.512247782703097</v>
       </c>
       <c r="BK2" t="n">
         <v>9</v>
@@ -1511,16 +1511,16 @@
         <v>1.691379759687266</v>
       </c>
       <c r="AP5" t="n">
-        <v>25.72727272727273</v>
+        <v>24.81818181818182</v>
       </c>
       <c r="AQ5" t="n">
-        <v>179.6363636363636</v>
+        <v>178</v>
       </c>
       <c r="AR5" t="n">
         <v>75.09090909090909</v>
       </c>
       <c r="AS5" t="n">
-        <v>-0.01912727705470375</v>
+        <v>0.08850406481472316</v>
       </c>
       <c r="AT5" t="n">
         <v>23.11111111111111</v>
@@ -1547,19 +1547,19 @@
         <v>-0.2417549780895007</v>
       </c>
       <c r="BB5" t="n">
-        <v>26</v>
+        <v>25.57142857142857</v>
       </c>
       <c r="BC5" t="n">
-        <v>183.1666666666667</v>
+        <v>181.2857142857143</v>
       </c>
       <c r="BD5" t="n">
-        <v>79.83333333333333</v>
+        <v>79.42857142857143</v>
       </c>
       <c r="BE5" t="n">
-        <v>1.569856974304203</v>
+        <v>1.425645352046227</v>
       </c>
       <c r="BF5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BG5" t="n">
         <v>26.28571428571428</v>
@@ -2339,16 +2339,16 @@
         <v>2.96075142878757</v>
       </c>
       <c r="AP9" t="n">
-        <v>25.1</v>
+        <v>25.44444444444444</v>
       </c>
       <c r="AQ9" t="n">
-        <v>182.1</v>
+        <v>182.6666666666667</v>
       </c>
       <c r="AR9" t="n">
-        <v>69.09999999999999</v>
+        <v>68.66666666666667</v>
       </c>
       <c r="AS9" t="n">
-        <v>-0.4110366191934048</v>
+        <v>-0.4235177712763121</v>
       </c>
       <c r="AT9" t="n">
         <v>24.75</v>
@@ -2534,16 +2534,16 @@
         </is>
       </c>
       <c r="AL10" t="n">
-        <v>26.5</v>
+        <v>26.6</v>
       </c>
       <c r="AM10" t="n">
-        <v>182</v>
+        <v>181.8</v>
       </c>
       <c r="AN10" t="n">
-        <v>76.5</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.236234644417211</v>
+        <v>0.2434538197865018</v>
       </c>
       <c r="AP10" t="n">
         <v>24.81818181818182</v>
@@ -2558,16 +2558,16 @@
         <v>0.215824066782216</v>
       </c>
       <c r="AT10" t="n">
-        <v>24.22222222222222</v>
+        <v>24.375</v>
       </c>
       <c r="AU10" t="n">
-        <v>182.1111111111111</v>
+        <v>183.375</v>
       </c>
       <c r="AV10" t="n">
-        <v>73</v>
+        <v>72.375</v>
       </c>
       <c r="AW10" t="n">
-        <v>-0.008535507131577556</v>
+        <v>-0.1247692438933886</v>
       </c>
       <c r="AX10" t="n">
         <v>24.42857142857143</v>
@@ -3203,34 +3203,34 @@
         <v>0.04758856804842998</v>
       </c>
       <c r="BB13" t="n">
-        <v>24.14285714285714</v>
+        <v>24.85714285714286</v>
       </c>
       <c r="BC13" t="n">
-        <v>176.8571428571429</v>
+        <v>178.2857142857143</v>
       </c>
       <c r="BD13" t="n">
-        <v>76.85714285714286</v>
+        <v>77.14285714285714</v>
       </c>
       <c r="BE13" t="n">
-        <v>0.5552190646631614</v>
+        <v>0.5706887261687845</v>
       </c>
       <c r="BF13" t="n">
         <v>7</v>
       </c>
       <c r="BG13" t="n">
-        <v>25.33333333333333</v>
+        <v>25.1</v>
       </c>
       <c r="BH13" t="n">
-        <v>183.3333333333333</v>
+        <v>182</v>
       </c>
       <c r="BI13" t="n">
-        <v>77.88888888888889</v>
+        <v>77.8</v>
       </c>
       <c r="BJ13" t="n">
-        <v>1.290113928744184</v>
+        <v>1.217140097719602</v>
       </c>
       <c r="BK13" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -3605,16 +3605,16 @@
         <v>-0.2869750904721419</v>
       </c>
       <c r="AX15" t="n">
-        <v>24.25</v>
+        <v>24.57142857142857</v>
       </c>
       <c r="AY15" t="n">
-        <v>180.625</v>
+        <v>181.5714285714286</v>
       </c>
       <c r="AZ15" t="n">
-        <v>72.625</v>
+        <v>72.42857142857143</v>
       </c>
       <c r="BA15" t="n">
-        <v>-0.06160145941209381</v>
+        <v>-0.1917077583666789</v>
       </c>
       <c r="BB15" t="n">
         <v>24.66666666666667</v>
@@ -4397,16 +4397,16 @@
         </is>
       </c>
       <c r="AL19" t="n">
-        <v>25</v>
+        <v>24.09090909090909</v>
       </c>
       <c r="AM19" t="n">
-        <v>180.8181818181818</v>
+        <v>179.1818181818182</v>
       </c>
       <c r="AN19" t="n">
         <v>74.36363636363636</v>
       </c>
       <c r="AO19" t="n">
-        <v>-0.1162580002051622</v>
+        <v>-0.008626658335735261</v>
       </c>
       <c r="AP19" t="n">
         <v>26.90909090909091</v>
@@ -5042,16 +5042,16 @@
         <v>0.6224605266742702</v>
       </c>
       <c r="AT22" t="n">
-        <v>25</v>
+        <v>25.16666666666667</v>
       </c>
       <c r="AU22" t="n">
-        <v>186.5</v>
+        <v>186.1666666666667</v>
       </c>
       <c r="AV22" t="n">
-        <v>74</v>
+        <v>74.66666666666667</v>
       </c>
       <c r="AW22" t="n">
-        <v>-0.06769263862993297</v>
+        <v>-0.05566067968111493</v>
       </c>
       <c r="AX22" t="n">
         <v>23.33333333333333</v>
@@ -5066,19 +5066,19 @@
         <v>1.118056915776086</v>
       </c>
       <c r="BB22" t="n">
-        <v>24.25</v>
+        <v>24.66666666666667</v>
       </c>
       <c r="BC22" t="n">
-        <v>171.5</v>
+        <v>171.3333333333333</v>
       </c>
       <c r="BD22" t="n">
-        <v>72.25</v>
+        <v>70.33333333333333</v>
       </c>
       <c r="BE22" t="n">
-        <v>0.03111982423723528</v>
+        <v>-0.2656183633379898</v>
       </c>
       <c r="BF22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BG22" t="n">
         <v>23</v>
@@ -5858,16 +5858,16 @@
         <v>-0.07819325734890144</v>
       </c>
       <c r="AP26" t="n">
-        <v>25.90909090909091</v>
+        <v>25</v>
       </c>
       <c r="AQ26" t="n">
-        <v>182.7272727272727</v>
+        <v>181.0909090909091</v>
       </c>
       <c r="AR26" t="n">
         <v>74.54545454545455</v>
       </c>
       <c r="AS26" t="n">
-        <v>-0.145790990352261</v>
+        <v>-0.0381596484828341</v>
       </c>
       <c r="AT26" t="n">
         <v>25.88888888888889</v>
@@ -6101,19 +6101,19 @@
         <v>-0.3580066195521284</v>
       </c>
       <c r="BB27" t="n">
-        <v>25.85714285714286</v>
+        <v>25.5</v>
       </c>
       <c r="BC27" t="n">
-        <v>184.2857142857143</v>
+        <v>182.5</v>
       </c>
       <c r="BD27" t="n">
-        <v>77.28571428571429</v>
+        <v>77.25</v>
       </c>
       <c r="BE27" t="n">
-        <v>1.204687020207576</v>
+        <v>1.124148094993925</v>
       </c>
       <c r="BF27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BG27" t="n">
         <v>32</v>
@@ -6503,16 +6503,16 @@
         <v>-0.01828640719634883</v>
       </c>
       <c r="AX29" t="n">
-        <v>25.55555555555556</v>
+        <v>26</v>
       </c>
       <c r="AY29" t="n">
-        <v>177.2222222222222</v>
+        <v>177.25</v>
       </c>
       <c r="AZ29" t="n">
-        <v>71.22222222222223</v>
+        <v>71</v>
       </c>
       <c r="BA29" t="n">
-        <v>-0.3789193101060265</v>
+        <v>-0.3889459425633748</v>
       </c>
       <c r="BB29" t="n">
         <v>27.28571428571428</v>
@@ -6737,16 +6737,16 @@
         <v>6</v>
       </c>
       <c r="BG30" t="n">
-        <v>24</v>
+        <v>24.71428571428572</v>
       </c>
       <c r="BH30" t="n">
-        <v>176.4285714285714</v>
+        <v>177.8571428571429</v>
       </c>
       <c r="BI30" t="n">
-        <v>76.71428571428571</v>
+        <v>77</v>
       </c>
       <c r="BJ30" t="n">
-        <v>0.4933404186406687</v>
+        <v>0.5088100801462918</v>
       </c>
       <c r="BK30" t="n">
         <v>7</v>
@@ -7151,16 +7151,16 @@
         <v>5</v>
       </c>
       <c r="BG32" t="n">
-        <v>22.83333333333333</v>
+        <v>23.66666666666667</v>
       </c>
       <c r="BH32" t="n">
-        <v>175.1666666666667</v>
+        <v>176.8333333333333</v>
       </c>
       <c r="BI32" t="n">
-        <v>76.5</v>
+        <v>76.83333333333333</v>
       </c>
       <c r="BJ32" t="n">
-        <v>0.5543596390239602</v>
+        <v>0.5724075774471872</v>
       </c>
       <c r="BK32" t="n">
         <v>6</v>
@@ -7538,16 +7538,16 @@
         <v>-0.00632964799096091</v>
       </c>
       <c r="AX34" t="n">
-        <v>23.55555555555556</v>
+        <v>23.66666666666667</v>
       </c>
       <c r="AY34" t="n">
-        <v>185.8888888888889</v>
+        <v>185.6666666666667</v>
       </c>
       <c r="AZ34" t="n">
-        <v>72.44444444444444</v>
+        <v>72.88888888888889</v>
       </c>
       <c r="BA34" t="n">
-        <v>-0.1035879828272401</v>
+        <v>-0.09556667686136144</v>
       </c>
       <c r="BB34" t="n">
         <v>33</v>
@@ -7565,19 +7565,19 @@
         <v>1</v>
       </c>
       <c r="BG34" t="n">
-        <v>24</v>
+        <v>24.5</v>
       </c>
       <c r="BH34" t="n">
-        <v>171.3333333333333</v>
+        <v>171</v>
       </c>
       <c r="BI34" t="n">
-        <v>71.33333333333333</v>
+        <v>68</v>
       </c>
       <c r="BJ34" t="n">
-        <v>0.04721256933127937</v>
+        <v>-0.3898483394845362</v>
       </c>
       <c r="BK34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -7912,16 +7912,16 @@
         </is>
       </c>
       <c r="AL36" t="n">
-        <v>25.45454545454545</v>
+        <v>24.54545454545455</v>
       </c>
       <c r="AM36" t="n">
-        <v>180.2727272727273</v>
+        <v>178.6363636363636</v>
       </c>
       <c r="AN36" t="n">
         <v>74.81818181818181</v>
       </c>
       <c r="AO36" t="n">
-        <v>-0.08016212335870802</v>
+        <v>0.02746921851071888</v>
       </c>
       <c r="AP36" t="n">
         <v>26</v>
@@ -8155,16 +8155,16 @@
         <v>1.485031663715036</v>
       </c>
       <c r="AX37" t="n">
-        <v>25</v>
+        <v>25.375</v>
       </c>
       <c r="AY37" t="n">
-        <v>179.5555555555555</v>
+        <v>179.875</v>
       </c>
       <c r="AZ37" t="n">
-        <v>69.11111111111111</v>
+        <v>68.625</v>
       </c>
       <c r="BA37" t="n">
-        <v>-0.4366727130603532</v>
+        <v>-0.4539185208869923</v>
       </c>
       <c r="BB37" t="n">
         <v>22.625</v>
@@ -8803,19 +8803,19 @@
         <v>3</v>
       </c>
       <c r="BG40" t="n">
-        <v>26</v>
+        <v>25.625</v>
       </c>
       <c r="BH40" t="n">
-        <v>183.5714285714286</v>
+        <v>181.875</v>
       </c>
       <c r="BI40" t="n">
-        <v>77.42857142857143</v>
+        <v>77.375</v>
       </c>
       <c r="BJ40" t="n">
-        <v>1.251096004724445</v>
+        <v>1.164755956446186</v>
       </c>
       <c r="BK40" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41">
@@ -8995,19 +8995,19 @@
         <v>-0.148106230937867</v>
       </c>
       <c r="BB41" t="n">
-        <v>26.28571428571428</v>
+        <v>25.875</v>
       </c>
       <c r="BC41" t="n">
-        <v>185.1428571428571</v>
+        <v>183.25</v>
       </c>
       <c r="BD41" t="n">
-        <v>76.85714285714286</v>
+        <v>76.875</v>
       </c>
       <c r="BE41" t="n">
-        <v>1.039677297480928</v>
+        <v>0.9797645876081083</v>
       </c>
       <c r="BF41" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BG41" t="n">
         <v>26</v>
@@ -10030,16 +10030,16 @@
         <v>-0.04362872073229687</v>
       </c>
       <c r="BB46" t="n">
-        <v>24.14285714285714</v>
+        <v>24.85714285714286</v>
       </c>
       <c r="BC46" t="n">
-        <v>176.5714285714286</v>
+        <v>178</v>
       </c>
       <c r="BD46" t="n">
-        <v>76.28571428571429</v>
+        <v>76.57142857142857</v>
       </c>
       <c r="BE46" t="n">
-        <v>0.4376496372204252</v>
+        <v>0.4531192987260483</v>
       </c>
       <c r="BF46" t="n">
         <v>7</v>
@@ -10201,16 +10201,16 @@
         <v>1.292137485476485</v>
       </c>
       <c r="AP47" t="n">
-        <v>25.45454545454545</v>
+        <v>24.54545454545455</v>
       </c>
       <c r="AQ47" t="n">
-        <v>180.2727272727273</v>
+        <v>178.6363636363636</v>
       </c>
       <c r="AR47" t="n">
         <v>74.81818181818181</v>
       </c>
       <c r="AS47" t="n">
-        <v>-0.08016212335870802</v>
+        <v>0.02746921851071888</v>
       </c>
       <c r="AT47" t="n">
         <v>25.5</v>
@@ -10420,16 +10420,16 @@
         <v>0.01027445535840799</v>
       </c>
       <c r="AT48" t="n">
-        <v>23.28571428571428</v>
+        <v>23.5</v>
       </c>
       <c r="AU48" t="n">
-        <v>179.4285714285714</v>
+        <v>179.8333333333333</v>
       </c>
       <c r="AV48" t="n">
-        <v>68.28571428571429</v>
+        <v>67.5</v>
       </c>
       <c r="AW48" t="n">
-        <v>-0.4263309578686309</v>
+        <v>-0.4476017424388628</v>
       </c>
       <c r="AX48" t="n">
         <v>22.71428571428572</v>
@@ -10627,16 +10627,16 @@
         <v>-0.05850459725083555</v>
       </c>
       <c r="AT49" t="n">
-        <v>24.5</v>
+        <v>24.625</v>
       </c>
       <c r="AU49" t="n">
-        <v>184.875</v>
+        <v>184.625</v>
       </c>
       <c r="AV49" t="n">
-        <v>73.375</v>
+        <v>73.875</v>
       </c>
       <c r="AW49" t="n">
-        <v>-0.1037885154763871</v>
+        <v>-0.09476454626477357</v>
       </c>
       <c r="AX49" t="n">
         <v>26.88888888888889</v>
@@ -10651,19 +10651,19 @@
         <v>0.253159600005215</v>
       </c>
       <c r="BB49" t="n">
-        <v>23.5</v>
+        <v>23.66666666666667</v>
       </c>
       <c r="BC49" t="n">
-        <v>173.5</v>
+        <v>174</v>
       </c>
       <c r="BD49" t="n">
-        <v>72.5</v>
+        <v>70.66666666666667</v>
       </c>
       <c r="BE49" t="n">
-        <v>0.06721570108368941</v>
+        <v>-0.2174905275427177</v>
       </c>
       <c r="BF49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BG49" t="n">
         <v>27.5</v>
@@ -11065,19 +11065,19 @@
         <v>-0.08453738115827823</v>
       </c>
       <c r="BB51" t="n">
-        <v>26.28571428571428</v>
+        <v>25.875</v>
       </c>
       <c r="BC51" t="n">
-        <v>185.1428571428571</v>
+        <v>183.25</v>
       </c>
       <c r="BD51" t="n">
-        <v>76.85714285714286</v>
+        <v>76.875</v>
       </c>
       <c r="BE51" t="n">
-        <v>1.039677297480928</v>
+        <v>0.9797645876081083</v>
       </c>
       <c r="BF51" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BG51" t="n">
         <v>31.5</v>
@@ -11893,16 +11893,16 @@
         <v>-0.2357962936577051</v>
       </c>
       <c r="BB55" t="n">
-        <v>25.22222222222222</v>
+        <v>25.77777777777778</v>
       </c>
       <c r="BC55" t="n">
-        <v>178.4444444444445</v>
+        <v>179.5555555555555</v>
       </c>
       <c r="BD55" t="n">
-        <v>77</v>
+        <v>77.22222222222223</v>
       </c>
       <c r="BE55" t="n">
-        <v>0.468932730487352</v>
+        <v>0.4809646894361699</v>
       </c>
       <c r="BF55" t="n">
         <v>9</v>
@@ -12064,16 +12064,16 @@
         <v>0.249294788948928</v>
       </c>
       <c r="AP56" t="n">
-        <v>25.45454545454545</v>
+        <v>24.54545454545455</v>
       </c>
       <c r="AQ56" t="n">
-        <v>179.8181818181818</v>
+        <v>178.1818181818182</v>
       </c>
       <c r="AR56" t="n">
         <v>75.09090909090909</v>
       </c>
       <c r="AS56" t="n">
-        <v>-0.001407482966444441</v>
+        <v>0.1062238589029825</v>
       </c>
       <c r="AT56" t="n">
         <v>26.875</v>
@@ -12490,16 +12490,16 @@
         <v>2.701189259828068</v>
       </c>
       <c r="AT58" t="n">
-        <v>25.11111111111111</v>
+        <v>25.5</v>
       </c>
       <c r="AU58" t="n">
-        <v>177.8888888888889</v>
+        <v>178</v>
       </c>
       <c r="AV58" t="n">
-        <v>69.22222222222223</v>
+        <v>68.75</v>
       </c>
       <c r="AW58" t="n">
-        <v>-0.4292530050419153</v>
+        <v>-0.4455713493662498</v>
       </c>
       <c r="AX58" t="n">
         <v>23.22222222222222</v>
@@ -12904,16 +12904,16 @@
         <v>-0.2906849444813608</v>
       </c>
       <c r="AT60" t="n">
-        <v>24.375</v>
+        <v>24.5</v>
       </c>
       <c r="AU60" t="n">
-        <v>185.625</v>
+        <v>185.375</v>
       </c>
       <c r="AV60" t="n">
-        <v>72.25</v>
+        <v>72.75</v>
       </c>
       <c r="AW60" t="n">
-        <v>-0.1189036639058398</v>
+        <v>-0.1098796946942262</v>
       </c>
       <c r="AX60" t="n">
         <v>23.77777777777778</v>
@@ -12928,19 +12928,19 @@
         <v>-0.08052672817533886</v>
       </c>
       <c r="BB60" t="n">
-        <v>24.8</v>
+        <v>25.25</v>
       </c>
       <c r="BC60" t="n">
-        <v>177.2</v>
+        <v>178.5</v>
       </c>
       <c r="BD60" t="n">
-        <v>73.8</v>
+        <v>72.75</v>
       </c>
       <c r="BE60" t="n">
-        <v>0.1008751062430079</v>
+        <v>-0.1042397139369678</v>
       </c>
       <c r="BF60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BG60" t="n">
         <v>27.66666666666667</v>
@@ -13150,19 +13150,19 @@
         <v>2</v>
       </c>
       <c r="BG61" t="n">
-        <v>25</v>
+        <v>24.77777777777778</v>
       </c>
       <c r="BH61" t="n">
-        <v>184.625</v>
+        <v>183</v>
       </c>
       <c r="BI61" t="n">
-        <v>77.375</v>
+        <v>77.33333333333333</v>
       </c>
       <c r="BJ61" t="n">
-        <v>1.277555571591355</v>
+        <v>1.197868910136579</v>
       </c>
       <c r="BK61" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="62">
@@ -13294,16 +13294,16 @@
         </is>
       </c>
       <c r="AL62" t="n">
-        <v>25.45454545454545</v>
+        <v>24.54545454545455</v>
       </c>
       <c r="AM62" t="n">
-        <v>180.2727272727273</v>
+        <v>178.6363636363636</v>
       </c>
       <c r="AN62" t="n">
         <v>74.81818181818181</v>
       </c>
       <c r="AO62" t="n">
-        <v>-0.08016212335870802</v>
+        <v>0.02746921851071888</v>
       </c>
       <c r="AP62" t="n">
         <v>26.72727272727273</v>
@@ -13564,16 +13564,16 @@
         <v>10</v>
       </c>
       <c r="BG63" t="n">
-        <v>25.22222222222222</v>
+        <v>25.77777777777778</v>
       </c>
       <c r="BH63" t="n">
-        <v>178.4444444444445</v>
+        <v>179.5555555555555</v>
       </c>
       <c r="BI63" t="n">
-        <v>77</v>
+        <v>77.22222222222223</v>
       </c>
       <c r="BJ63" t="n">
-        <v>0.468932730487352</v>
+        <v>0.4809646894361699</v>
       </c>
       <c r="BK63" t="n">
         <v>9</v>
@@ -14544,16 +14544,16 @@
         <v>3.224907618436621</v>
       </c>
       <c r="AP68" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="AQ68" t="n">
-        <v>182.5</v>
+        <v>182.3</v>
       </c>
       <c r="AR68" t="n">
-        <v>75.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="AS68" t="n">
-        <v>0.1106209929915505</v>
+        <v>0.1178401683608414</v>
       </c>
       <c r="AT68" t="n">
         <v>25.71428571428572</v>
@@ -14595,19 +14595,19 @@
         <v>4</v>
       </c>
       <c r="BG68" t="n">
-        <v>23.2</v>
+        <v>23.25</v>
       </c>
       <c r="BH68" t="n">
-        <v>176.8</v>
+        <v>178</v>
       </c>
       <c r="BI68" t="n">
-        <v>73.8</v>
+        <v>72.75</v>
       </c>
       <c r="BJ68" t="n">
-        <v>0.2683599748105551</v>
+        <v>0.1051163717724663</v>
       </c>
       <c r="BK68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69">
@@ -14958,16 +14958,16 @@
         <v>-0.29238947199911</v>
       </c>
       <c r="AP70" t="n">
-        <v>27.09090909090909</v>
+        <v>27.6</v>
       </c>
       <c r="AQ70" t="n">
-        <v>180.3636363636364</v>
+        <v>180.7</v>
       </c>
       <c r="AR70" t="n">
-        <v>73.09090909090909</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="AS70" t="n">
-        <v>-0.2973936731073684</v>
+        <v>-0.2972624153733813</v>
       </c>
       <c r="AT70" t="n">
         <v>24.33333333333333</v>
@@ -15189,16 +15189,16 @@
         <v>-0.09496507891392053</v>
       </c>
       <c r="AX71" t="n">
-        <v>25.22222222222222</v>
+        <v>25.33333333333333</v>
       </c>
       <c r="AY71" t="n">
-        <v>182.3333333333333</v>
+        <v>182.1111111111111</v>
       </c>
       <c r="AZ71" t="n">
-        <v>73.33333333333333</v>
+        <v>73.77777777777777</v>
       </c>
       <c r="BA71" t="n">
-        <v>-0.1791887915556468</v>
+        <v>-0.1711674855897682</v>
       </c>
       <c r="BB71" t="n">
         <v>25.5</v>
@@ -15216,19 +15216,19 @@
         <v>4</v>
       </c>
       <c r="BG71" t="n">
-        <v>25.33333333333333</v>
+        <v>26.5</v>
       </c>
       <c r="BH71" t="n">
-        <v>177.3333333333333</v>
+        <v>180</v>
       </c>
       <c r="BI71" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="BJ71" t="n">
-        <v>0.04961896112104299</v>
+        <v>-0.3862387517998908</v>
       </c>
       <c r="BK71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -15615,19 +15615,19 @@
         <v>0.2670966191209292</v>
       </c>
       <c r="BB73" t="n">
-        <v>25.125</v>
+        <v>24.88888888888889</v>
       </c>
       <c r="BC73" t="n">
-        <v>183.875</v>
+        <v>182.3333333333333</v>
       </c>
       <c r="BD73" t="n">
-        <v>76.75</v>
+        <v>76.77777777777777</v>
       </c>
       <c r="BE73" t="n">
-        <v>0.9887885568197217</v>
+        <v>0.9411871192284603</v>
       </c>
       <c r="BF73" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BG73" t="n">
         <v>26.5</v>
@@ -16665,16 +16665,16 @@
         <v>2</v>
       </c>
       <c r="BG78" t="n">
-        <v>26.875</v>
+        <v>27.5</v>
       </c>
       <c r="BH78" t="n">
-        <v>179.125</v>
+        <v>180.375</v>
       </c>
       <c r="BI78" t="n">
-        <v>76.875</v>
+        <v>77.125</v>
       </c>
       <c r="BJ78" t="n">
-        <v>0.3519219297100964</v>
+        <v>0.3654578835275167</v>
       </c>
       <c r="BK78" t="n">
         <v>8</v>
@@ -16809,28 +16809,28 @@
         </is>
       </c>
       <c r="AL79" t="n">
-        <v>25.8</v>
+        <v>26.22222222222222</v>
       </c>
       <c r="AM79" t="n">
-        <v>178.6</v>
+        <v>178.7777777777778</v>
       </c>
       <c r="AN79" t="n">
-        <v>72.90000000000001</v>
+        <v>72.88888888888889</v>
       </c>
       <c r="AO79" t="n">
-        <v>-0.3225295291658993</v>
+        <v>-0.3251765601346392</v>
       </c>
       <c r="AP79" t="n">
-        <v>25.90909090909091</v>
+        <v>25</v>
       </c>
       <c r="AQ79" t="n">
-        <v>181.5454545454545</v>
+        <v>179.9090909090909</v>
       </c>
       <c r="AR79" t="n">
         <v>74.72727272727273</v>
       </c>
       <c r="AS79" t="n">
-        <v>-0.1228208869045175</v>
+        <v>-0.01518954503509057</v>
       </c>
       <c r="AT79" t="n">
         <v>25.22222222222222</v>
@@ -17649,16 +17649,16 @@
         <v>0.1252562303311129</v>
       </c>
       <c r="AP83" t="n">
-        <v>25.8</v>
+        <v>26.22222222222222</v>
       </c>
       <c r="AQ83" t="n">
-        <v>178.6</v>
+        <v>178.7777777777778</v>
       </c>
       <c r="AR83" t="n">
-        <v>72.90000000000001</v>
+        <v>72.88888888888889</v>
       </c>
       <c r="AS83" t="n">
-        <v>-0.3225295291658992</v>
+        <v>-0.3251765601346392</v>
       </c>
       <c r="AT83" t="n">
         <v>22.71428571428572</v>
@@ -17685,16 +17685,16 @@
         <v>-0.4752551947562297</v>
       </c>
       <c r="BB83" t="n">
-        <v>27</v>
+        <v>27.71428571428572</v>
       </c>
       <c r="BC83" t="n">
-        <v>176.2857142857143</v>
+        <v>177.7142857142857</v>
       </c>
       <c r="BD83" t="n">
-        <v>76.57142857142857</v>
+        <v>76.85714285714286</v>
       </c>
       <c r="BE83" t="n">
-        <v>0.2086986469372016</v>
+        <v>0.2241683084428249</v>
       </c>
       <c r="BF83" t="n">
         <v>7</v>
@@ -18248,16 +18248,16 @@
         </is>
       </c>
       <c r="AL86" t="n">
-        <v>25.09090909090909</v>
+        <v>24.18181818181818</v>
       </c>
       <c r="AM86" t="n">
-        <v>180.7272727272727</v>
+        <v>179.0909090909091</v>
       </c>
       <c r="AN86" t="n">
         <v>74.63636363636364</v>
       </c>
       <c r="AO86" t="n">
-        <v>-0.1136328455254201</v>
+        <v>-0.006001503655993157</v>
       </c>
       <c r="AP86" t="n">
         <v>25.72727272727273</v>
@@ -19100,16 +19100,16 @@
         <v>1.632423160838057</v>
       </c>
       <c r="AT90" t="n">
-        <v>25.22222222222222</v>
+        <v>25.33333333333333</v>
       </c>
       <c r="AU90" t="n">
-        <v>182.3333333333333</v>
+        <v>182.1111111111111</v>
       </c>
       <c r="AV90" t="n">
-        <v>73.33333333333333</v>
+        <v>73.77777777777777</v>
       </c>
       <c r="AW90" t="n">
-        <v>-0.1791887915556468</v>
+        <v>-0.1711674855897682</v>
       </c>
       <c r="AX90" t="n">
         <v>22.77777777777778</v>
@@ -19124,34 +19124,34 @@
         <v>0.3411934329807337</v>
       </c>
       <c r="BB90" t="n">
-        <v>21.5</v>
+        <v>20</v>
       </c>
       <c r="BC90" t="n">
         <v>172</v>
       </c>
       <c r="BD90" t="n">
-        <v>69.5</v>
+        <v>61</v>
       </c>
       <c r="BE90" t="n">
-        <v>0.1912952777433755</v>
+        <v>-0.5387438314761596</v>
       </c>
       <c r="BF90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BG90" t="n">
-        <v>25.83333333333333</v>
+        <v>25.42857142857143</v>
       </c>
       <c r="BH90" t="n">
-        <v>184.1666666666667</v>
+        <v>182.1428571428571</v>
       </c>
       <c r="BI90" t="n">
-        <v>76.5</v>
+        <v>76.57142857142857</v>
       </c>
       <c r="BJ90" t="n">
-        <v>1.065417095375007</v>
+        <v>0.9932683129640585</v>
       </c>
       <c r="BK90" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91">
@@ -19331,19 +19331,19 @@
         <v>0.5363117006007331</v>
       </c>
       <c r="BB91" t="n">
-        <v>27.75</v>
+        <v>26.8</v>
       </c>
       <c r="BC91" t="n">
-        <v>183.5</v>
+        <v>180.8</v>
       </c>
       <c r="BD91" t="n">
-        <v>73</v>
+        <v>73.8</v>
       </c>
       <c r="BE91" t="n">
-        <v>-0.1980889937377486</v>
+        <v>-0.04639607129052502</v>
       </c>
       <c r="BF91" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BG91" t="n">
         <v>23.25</v>
@@ -20588,16 +20588,16 @@
         <v>2</v>
       </c>
       <c r="BG97" t="n">
-        <v>24.66666666666667</v>
+        <v>26.33333333333333</v>
       </c>
       <c r="BH97" t="n">
-        <v>176.3333333333333</v>
+        <v>179.6666666666667</v>
       </c>
       <c r="BI97" t="n">
-        <v>74.33333333333333</v>
+        <v>75</v>
       </c>
       <c r="BJ97" t="n">
-        <v>-0.002720060306315497</v>
+        <v>0.03337581654013864</v>
       </c>
       <c r="BK97" t="n">
         <v>3</v>
@@ -20795,16 +20795,16 @@
         <v>1</v>
       </c>
       <c r="BG98" t="n">
-        <v>29.5</v>
+        <v>27.83333333333333</v>
       </c>
       <c r="BH98" t="n">
-        <v>181.8333333333333</v>
+        <v>178.8333333333333</v>
       </c>
       <c r="BI98" t="n">
         <v>74</v>
       </c>
       <c r="BJ98" t="n">
-        <v>-0.2752439304970443</v>
+        <v>-0.07791980373642832</v>
       </c>
       <c r="BK98" t="n">
         <v>6</v>
@@ -20939,28 +20939,28 @@
         </is>
       </c>
       <c r="AL99" t="n">
-        <v>26.1</v>
+        <v>26.55555555555556</v>
       </c>
       <c r="AM99" t="n">
-        <v>178.6</v>
+        <v>178.7777777777778</v>
       </c>
       <c r="AN99" t="n">
-        <v>72.7</v>
+        <v>72.66666666666667</v>
       </c>
       <c r="AO99" t="n">
-        <v>-0.3283048694613319</v>
+        <v>-0.3315936049073421</v>
       </c>
       <c r="AP99" t="n">
-        <v>26.6</v>
+        <v>26.7</v>
       </c>
       <c r="AQ99" t="n">
-        <v>185.4</v>
+        <v>185.2</v>
       </c>
       <c r="AR99" t="n">
-        <v>76.7</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="AS99" t="n">
-        <v>0.2434538197865018</v>
+        <v>0.2506729951557926</v>
       </c>
       <c r="AT99" t="n">
         <v>22.44444444444444</v>
@@ -21002,19 +21002,19 @@
         <v>8</v>
       </c>
       <c r="BG99" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="BH99" t="n">
-        <v>174.6666666666667</v>
+        <v>176</v>
       </c>
       <c r="BI99" t="n">
-        <v>70.66666666666667</v>
+        <v>67</v>
       </c>
       <c r="BJ99" t="n">
-        <v>0.08571483796749713</v>
+        <v>-0.3320949365302096</v>
       </c>
       <c r="BK99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="100">
@@ -21815,16 +21815,16 @@
         <v>-0.1223521092831349</v>
       </c>
       <c r="BB103" t="n">
-        <v>24</v>
+        <v>25.25</v>
       </c>
       <c r="BC103" t="n">
-        <v>173</v>
+        <v>175.5</v>
       </c>
       <c r="BD103" t="n">
-        <v>74.5</v>
+        <v>75</v>
       </c>
       <c r="BE103" t="n">
-        <v>-0.006329647990960904</v>
+        <v>0.0207422596438797</v>
       </c>
       <c r="BF103" t="n">
         <v>4</v>
@@ -22388,16 +22388,16 @@
         </is>
       </c>
       <c r="AL106" t="n">
-        <v>26.4</v>
+        <v>26.77777777777778</v>
       </c>
       <c r="AM106" t="n">
-        <v>183</v>
+        <v>184.2222222222222</v>
       </c>
       <c r="AN106" t="n">
-        <v>76.7</v>
+        <v>76.55555555555556</v>
       </c>
       <c r="AO106" t="n">
-        <v>0.2939880473715376</v>
+        <v>0.2242828985280517</v>
       </c>
       <c r="AP106" t="n">
         <v>28.36363636363636</v>
@@ -22412,16 +22412,16 @@
         <v>1.259323051979708</v>
       </c>
       <c r="AT106" t="n">
-        <v>25.77777777777778</v>
+        <v>25.88888888888889</v>
       </c>
       <c r="AU106" t="n">
-        <v>182.6666666666667</v>
+        <v>182.4444444444445</v>
       </c>
       <c r="AV106" t="n">
-        <v>74.66666666666667</v>
+        <v>75.11111111111111</v>
       </c>
       <c r="AW106" t="n">
-        <v>-0.007532843885842719</v>
+        <v>0.0004884620800359699</v>
       </c>
       <c r="AX106" t="n">
         <v>27.22222222222222</v>
@@ -22607,16 +22607,16 @@
         <v>2.415703688406112</v>
       </c>
       <c r="AP107" t="n">
-        <v>25.2</v>
+        <v>25.55555555555556</v>
       </c>
       <c r="AQ107" t="n">
-        <v>180.3</v>
+        <v>180.6666666666667</v>
       </c>
       <c r="AR107" t="n">
-        <v>72</v>
+        <v>71.88888888888889</v>
       </c>
       <c r="AS107" t="n">
-        <v>-0.3333582922198355</v>
+        <v>-0.3372085190834572</v>
       </c>
       <c r="AT107" t="n">
         <v>25.25</v>
@@ -22850,16 +22850,16 @@
         <v>-0.1262481721808475</v>
       </c>
       <c r="BB108" t="n">
-        <v>28.2</v>
+        <v>26.2</v>
       </c>
       <c r="BC108" t="n">
-        <v>180.6</v>
+        <v>177</v>
       </c>
       <c r="BD108" t="n">
         <v>74.40000000000001</v>
       </c>
       <c r="BE108" t="n">
-        <v>-0.2149638161634659</v>
+        <v>0.02182513594927331</v>
       </c>
       <c r="BF108" t="n">
         <v>5</v>
@@ -23279,19 +23279,19 @@
         <v>4</v>
       </c>
       <c r="BG110" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="BH110" t="n">
-        <v>184.3333333333333</v>
+        <v>180.75</v>
       </c>
       <c r="BI110" t="n">
-        <v>71.66666666666667</v>
+        <v>73</v>
       </c>
       <c r="BJ110" t="n">
-        <v>-0.2704311469175171</v>
+        <v>-0.06272945556354552</v>
       </c>
       <c r="BK110" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="111">
@@ -23471,19 +23471,19 @@
         <v>-0.2256120998331698</v>
       </c>
       <c r="BB111" t="n">
-        <v>26.6</v>
+        <v>26</v>
       </c>
       <c r="BC111" t="n">
-        <v>184.4</v>
+        <v>182</v>
       </c>
       <c r="BD111" t="n">
-        <v>75.40000000000001</v>
+        <v>75.66666666666667</v>
       </c>
       <c r="BE111" t="n">
-        <v>0.5311379582527413</v>
+        <v>0.5360109016270126</v>
       </c>
       <c r="BF111" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BG111" t="n">
         <v>25.8</v>
@@ -23837,16 +23837,16 @@
         </is>
       </c>
       <c r="AL113" t="n">
-        <v>25.5</v>
+        <v>25.88888888888889</v>
       </c>
       <c r="AM113" t="n">
-        <v>180.2</v>
+        <v>180.5555555555555</v>
       </c>
       <c r="AN113" t="n">
         <v>73</v>
       </c>
       <c r="AO113" t="n">
-        <v>-0.3145884362596792</v>
+        <v>-0.3163531235721726</v>
       </c>
       <c r="AP113" t="n">
         <v>26.54545454545455</v>
@@ -24251,28 +24251,28 @@
         </is>
       </c>
       <c r="AL115" t="n">
-        <v>24.09090909090909</v>
+        <v>23.18181818181818</v>
       </c>
       <c r="AM115" t="n">
-        <v>182.6363636363636</v>
+        <v>181</v>
       </c>
       <c r="AN115" t="n">
         <v>74.63636363636364</v>
       </c>
       <c r="AO115" t="n">
-        <v>-0.09656934010709627</v>
+        <v>0.01106200176233063</v>
       </c>
       <c r="AP115" t="n">
-        <v>25.9</v>
+        <v>26.22222222222222</v>
       </c>
       <c r="AQ115" t="n">
-        <v>182.7</v>
+        <v>183.8888888888889</v>
       </c>
       <c r="AR115" t="n">
-        <v>76.09999999999999</v>
+        <v>75.88888888888889</v>
       </c>
       <c r="AS115" t="n">
-        <v>0.2405661496387854</v>
+        <v>0.1649252343805493</v>
       </c>
       <c r="AT115" t="n">
         <v>26.44444444444444</v>
@@ -24287,16 +24287,16 @@
         <v>-0.203252709453283</v>
       </c>
       <c r="AX115" t="n">
-        <v>24.11111111111111</v>
+        <v>24.22222222222222</v>
       </c>
       <c r="AY115" t="n">
-        <v>182.6666666666667</v>
+        <v>182.4444444444445</v>
       </c>
       <c r="AZ115" t="n">
-        <v>71.22222222222223</v>
+        <v>71.66666666666667</v>
       </c>
       <c r="BA115" t="n">
-        <v>-0.1575312654477743</v>
+        <v>-0.1495099594818957</v>
       </c>
       <c r="BB115" t="n">
         <v>27.33333333333333</v>
@@ -24677,16 +24677,16 @@
         <v>3.653792264239489</v>
       </c>
       <c r="AP117" t="n">
-        <v>27.18181818181818</v>
+        <v>27.63636363636364</v>
       </c>
       <c r="AQ117" t="n">
-        <v>180.9090909090909</v>
+        <v>181.8181818181818</v>
       </c>
       <c r="AR117" t="n">
-        <v>76</v>
+        <v>76.18181818181819</v>
       </c>
       <c r="AS117" t="n">
-        <v>0.1908850973246658</v>
+        <v>0.2007294273736988</v>
       </c>
       <c r="AT117" t="n">
         <v>25.55555555555556</v>
@@ -25700,16 +25700,16 @@
         </is>
       </c>
       <c r="AL122" t="n">
-        <v>24.27272727272727</v>
+        <v>24.72727272727273</v>
       </c>
       <c r="AM122" t="n">
-        <v>182.5454545454545</v>
+        <v>183.4545454545455</v>
       </c>
       <c r="AN122" t="n">
-        <v>76.18181818181819</v>
+        <v>76.36363636363636</v>
       </c>
       <c r="AO122" t="n">
-        <v>0.3293620066810626</v>
+        <v>0.3392063367300956</v>
       </c>
       <c r="AP122" t="n">
         <v>26.54545454545455</v>
@@ -26114,16 +26114,16 @@
         </is>
       </c>
       <c r="AL124" t="n">
-        <v>26.5</v>
+        <v>26.88888888888889</v>
       </c>
       <c r="AM124" t="n">
-        <v>182.3</v>
+        <v>183.4444444444445</v>
       </c>
       <c r="AN124" t="n">
-        <v>77.5</v>
+        <v>77.44444444444444</v>
       </c>
       <c r="AO124" t="n">
-        <v>0.3907249973200347</v>
+        <v>0.3317683984708262</v>
       </c>
       <c r="AP124" t="n">
         <v>26.45454545454545</v>
@@ -26138,16 +26138,16 @@
         <v>1.626844707143606</v>
       </c>
       <c r="AT124" t="n">
-        <v>25.66666666666667</v>
+        <v>25.77777777777778</v>
       </c>
       <c r="AU124" t="n">
-        <v>183.4444444444445</v>
+        <v>183.2222222222222</v>
       </c>
       <c r="AV124" t="n">
-        <v>73.77777777777777</v>
+        <v>74.22222222222223</v>
       </c>
       <c r="AW124" t="n">
-        <v>-0.1150183438286173</v>
+        <v>-0.1069970378627386</v>
       </c>
       <c r="AX124" t="n">
         <v>26.33333333333333</v>
@@ -26747,16 +26747,16 @@
         <v>0.217136644122087</v>
       </c>
       <c r="AP127" t="n">
-        <v>25.54545454545455</v>
+        <v>24.63636363636364</v>
       </c>
       <c r="AQ127" t="n">
-        <v>182.3636363636364</v>
+        <v>180.7272727272727</v>
       </c>
       <c r="AR127" t="n">
         <v>74.81818181818181</v>
       </c>
       <c r="AS127" t="n">
-        <v>-0.101163360796645</v>
+        <v>0.00646798107278193</v>
       </c>
       <c r="AT127" t="n">
         <v>23</v>
@@ -26954,16 +26954,16 @@
         <v>0.2729211810666071</v>
       </c>
       <c r="AP128" t="n">
-        <v>26.4</v>
+        <v>26.88888888888889</v>
       </c>
       <c r="AQ128" t="n">
-        <v>182.7</v>
+        <v>183.3333333333333</v>
       </c>
       <c r="AR128" t="n">
-        <v>73.59999999999999</v>
+        <v>73.66666666666667</v>
       </c>
       <c r="AS128" t="n">
-        <v>-0.2640542086746435</v>
+        <v>-0.2602039818110217</v>
       </c>
       <c r="AT128" t="n">
         <v>26.77777777777778</v>
@@ -27419,19 +27419,19 @@
         <v>5</v>
       </c>
       <c r="BG130" t="n">
-        <v>25.8</v>
+        <v>25.33333333333333</v>
       </c>
       <c r="BH130" t="n">
-        <v>183.8</v>
+        <v>181.5</v>
       </c>
       <c r="BI130" t="n">
-        <v>74.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="BJ130" t="n">
-        <v>0.3867544508669248</v>
+        <v>0.4156913121388321</v>
       </c>
       <c r="BK130" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131">
@@ -28208,16 +28208,16 @@
         <v>2.854104519923046</v>
       </c>
       <c r="AT134" t="n">
-        <v>24.14285714285714</v>
+        <v>24</v>
       </c>
       <c r="AU134" t="n">
-        <v>185.8571428571429</v>
+        <v>183.875</v>
       </c>
       <c r="AV134" t="n">
-        <v>73</v>
+        <v>73.5</v>
       </c>
       <c r="AW134" t="n">
-        <v>0.2450523514754162</v>
+        <v>0.2844677598532853</v>
       </c>
       <c r="AX134" t="n">
         <v>24.25</v>
@@ -28391,16 +28391,16 @@
         </is>
       </c>
       <c r="AL135" t="n">
-        <v>25</v>
+        <v>24.09090909090909</v>
       </c>
       <c r="AM135" t="n">
-        <v>181</v>
+        <v>179.3636363636364</v>
       </c>
       <c r="AN135" t="n">
         <v>75.18181818181819</v>
       </c>
       <c r="AO135" t="n">
-        <v>-0.02306500907431691</v>
+        <v>0.08456633279510997</v>
       </c>
       <c r="AP135" t="n">
         <v>24.3</v>
@@ -29231,16 +29231,16 @@
         <v>0.6614440736684408</v>
       </c>
       <c r="AP139" t="n">
-        <v>25.3</v>
+        <v>25.66666666666667</v>
       </c>
       <c r="AQ139" t="n">
-        <v>181.6</v>
+        <v>182.1111111111111</v>
       </c>
       <c r="AR139" t="n">
-        <v>73.2</v>
+        <v>73.22222222222223</v>
       </c>
       <c r="AS139" t="n">
-        <v>-0.2582788683792109</v>
+        <v>-0.2537869370383188</v>
       </c>
       <c r="AT139" t="n">
         <v>28.44444444444444</v>
@@ -29426,16 +29426,16 @@
         </is>
       </c>
       <c r="AL140" t="n">
-        <v>26.5</v>
+        <v>26.88888888888889</v>
       </c>
       <c r="AM140" t="n">
-        <v>182.3</v>
+        <v>183.4444444444445</v>
       </c>
       <c r="AN140" t="n">
-        <v>77.5</v>
+        <v>77.44444444444444</v>
       </c>
       <c r="AO140" t="n">
-        <v>0.3907249973200347</v>
+        <v>0.3317683984708262</v>
       </c>
       <c r="AP140" t="n">
         <v>25.90909090909091</v>
@@ -29474,16 +29474,16 @@
         <v>0.7478936987156984</v>
       </c>
       <c r="BB140" t="n">
-        <v>23</v>
+        <v>23.5</v>
       </c>
       <c r="BC140" t="n">
-        <v>175.5</v>
+        <v>174.5</v>
       </c>
       <c r="BD140" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="BE140" t="n">
-        <v>-0.1940282075925225</v>
+        <v>-0.1579323307460683</v>
       </c>
       <c r="BF140" t="n">
         <v>2</v>
@@ -29645,16 +29645,16 @@
         <v>1.669503470689415</v>
       </c>
       <c r="AP141" t="n">
-        <v>26</v>
+        <v>26.45454545454545</v>
       </c>
       <c r="AQ141" t="n">
-        <v>181.7272727272727</v>
+        <v>182.6363636363636</v>
       </c>
       <c r="AR141" t="n">
-        <v>75.45454545454545</v>
+        <v>75.63636363636364</v>
       </c>
       <c r="AS141" t="n">
-        <v>0.2794840677659624</v>
+        <v>0.2893283978149953</v>
       </c>
       <c r="AT141" t="n">
         <v>26.77777777777778</v>
@@ -29840,16 +29840,16 @@
         </is>
       </c>
       <c r="AL142" t="n">
-        <v>25.8</v>
+        <v>26.22222222222222</v>
       </c>
       <c r="AM142" t="n">
-        <v>180</v>
+        <v>180.3333333333333</v>
       </c>
       <c r="AN142" t="n">
-        <v>73.40000000000001</v>
+        <v>73.44444444444444</v>
       </c>
       <c r="AO142" t="n">
-        <v>-0.2575569508422818</v>
+        <v>-0.2529848064417309</v>
       </c>
       <c r="AP142" t="n">
         <v>27.54545454545455</v>
@@ -30083,16 +30083,16 @@
         <v>0.8121443595023868</v>
       </c>
       <c r="AX143" t="n">
-        <v>26.85714285714286</v>
+        <v>26.375</v>
       </c>
       <c r="AY143" t="n">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AZ143" t="n">
-        <v>77.85714285714286</v>
+        <v>77.75</v>
       </c>
       <c r="BA143" t="n">
-        <v>0.602917187638833</v>
+        <v>0.597599491496275</v>
       </c>
       <c r="BB143" t="n">
         <v>25.5</v>
@@ -30266,28 +30266,28 @@
         <v>0.2112300460926672</v>
       </c>
       <c r="AP144" t="n">
-        <v>24.81818181818182</v>
+        <v>23.90909090909091</v>
       </c>
       <c r="AQ144" t="n">
-        <v>181.6363636363636</v>
+        <v>180</v>
       </c>
       <c r="AR144" t="n">
         <v>75</v>
       </c>
       <c r="AS144" t="n">
-        <v>-0.04275366917238282</v>
+        <v>0.06487767269704409</v>
       </c>
       <c r="AT144" t="n">
-        <v>24.77777777777778</v>
+        <v>25.33333333333333</v>
       </c>
       <c r="AU144" t="n">
-        <v>177.8888888888889</v>
+        <v>179</v>
       </c>
       <c r="AV144" t="n">
-        <v>75.44444444444444</v>
+        <v>75.66666666666667</v>
       </c>
       <c r="AW144" t="n">
-        <v>0.3109130029595416</v>
+        <v>0.3229449619083596</v>
       </c>
       <c r="AX144" t="n">
         <v>25.33333333333333</v>
@@ -31508,16 +31508,16 @@
         <v>-0.343990168672791</v>
       </c>
       <c r="AP150" t="n">
-        <v>26.36363636363636</v>
+        <v>26.7</v>
       </c>
       <c r="AQ150" t="n">
-        <v>181.3636363636364</v>
+        <v>182.3</v>
       </c>
       <c r="AR150" t="n">
-        <v>77.27272727272727</v>
+        <v>77.2</v>
       </c>
       <c r="AS150" t="n">
-        <v>0.3536446874686772</v>
+        <v>0.2968757175192539</v>
       </c>
       <c r="AT150" t="n">
         <v>26.55555555555556</v>
@@ -31532,16 +31532,16 @@
         <v>-0.4146141216541867</v>
       </c>
       <c r="AX150" t="n">
-        <v>24.75</v>
+        <v>24.875</v>
       </c>
       <c r="AY150" t="n">
-        <v>183.875</v>
+        <v>183.625</v>
       </c>
       <c r="AZ150" t="n">
-        <v>73.125</v>
+        <v>73.625</v>
       </c>
       <c r="BA150" t="n">
-        <v>-0.1714682845634886</v>
+        <v>-0.1624443153518751</v>
       </c>
       <c r="BB150" t="n">
         <v>27.75</v>
@@ -32324,16 +32324,16 @@
         </is>
       </c>
       <c r="AL154" t="n">
-        <v>24.54545454545455</v>
+        <v>23.63636363636364</v>
       </c>
       <c r="AM154" t="n">
-        <v>182.1818181818182</v>
+        <v>180.5454545454545</v>
       </c>
       <c r="AN154" t="n">
         <v>74.54545454545455</v>
       </c>
       <c r="AO154" t="n">
-        <v>-0.1116639795156135</v>
+        <v>-0.004032637646186558</v>
       </c>
       <c r="AP154" t="n">
         <v>24.5</v>
@@ -33359,28 +33359,28 @@
         </is>
       </c>
       <c r="AL159" t="n">
-        <v>24.55555555555556</v>
+        <v>24.4</v>
       </c>
       <c r="AM159" t="n">
-        <v>183.8888888888889</v>
+        <v>182.5</v>
       </c>
       <c r="AN159" t="n">
-        <v>81.77777777777777</v>
+        <v>81.3</v>
       </c>
       <c r="AO159" t="n">
-        <v>2.413297296616348</v>
+        <v>2.228005128804551</v>
       </c>
       <c r="AP159" t="n">
-        <v>25.7</v>
+        <v>26.11111111111111</v>
       </c>
       <c r="AQ159" t="n">
-        <v>182.1</v>
+        <v>182.6666666666667</v>
       </c>
       <c r="AR159" t="n">
-        <v>73.09999999999999</v>
+        <v>73.11111111111111</v>
       </c>
       <c r="AS159" t="n">
-        <v>-0.2763268068024379</v>
+        <v>-0.2738402019530155</v>
       </c>
       <c r="AT159" t="n">
         <v>28.125</v>
@@ -33763,16 +33763,16 @@
         </is>
       </c>
       <c r="AL161" t="n">
-        <v>26.36363636363636</v>
+        <v>26.7</v>
       </c>
       <c r="AM161" t="n">
-        <v>181.3636363636364</v>
+        <v>182.3</v>
       </c>
       <c r="AN161" t="n">
-        <v>77.27272727272727</v>
+        <v>77.2</v>
       </c>
       <c r="AO161" t="n">
-        <v>0.3536446874686772</v>
+        <v>0.2968757175192539</v>
       </c>
       <c r="AP161" t="n">
         <v>25.9</v>
@@ -33787,16 +33787,16 @@
         <v>2.34639960486092</v>
       </c>
       <c r="AT161" t="n">
-        <v>24.75</v>
+        <v>24.875</v>
       </c>
       <c r="AU161" t="n">
-        <v>183.875</v>
+        <v>183.625</v>
       </c>
       <c r="AV161" t="n">
-        <v>73.125</v>
+        <v>73.625</v>
       </c>
       <c r="AW161" t="n">
-        <v>-0.1714682845634886</v>
+        <v>-0.1624443153518751</v>
       </c>
       <c r="AX161" t="n">
         <v>23.77777777777778</v>
@@ -34189,16 +34189,16 @@
         <v>0.3871154096353893</v>
       </c>
       <c r="AP163" t="n">
-        <v>26.27272727272727</v>
+        <v>26.6</v>
       </c>
       <c r="AQ163" t="n">
-        <v>182.2727272727273</v>
+        <v>183.3</v>
       </c>
       <c r="AR163" t="n">
-        <v>77.09090909090909</v>
+        <v>77</v>
       </c>
       <c r="AS163" t="n">
-        <v>0.327393140671256</v>
+        <v>0.2679990160420906</v>
       </c>
       <c r="AT163" t="n">
         <v>26.22222222222222</v>
@@ -34591,16 +34591,16 @@
         </is>
       </c>
       <c r="AL165" t="n">
-        <v>24.72727272727273</v>
+        <v>25.18181818181818</v>
       </c>
       <c r="AM165" t="n">
-        <v>181.7272727272727</v>
+        <v>182.6363636363636</v>
       </c>
       <c r="AN165" t="n">
-        <v>76.81818181818181</v>
+        <v>77</v>
       </c>
       <c r="AO165" t="n">
-        <v>0.4087729357432617</v>
+        <v>0.4186172657922947</v>
       </c>
       <c r="AP165" t="n">
         <v>27.27272727272727</v>
@@ -34810,16 +34810,16 @@
         <v>0.2880158204751243</v>
       </c>
       <c r="AP166" t="n">
-        <v>24.90909090909091</v>
+        <v>24</v>
       </c>
       <c r="AQ166" t="n">
-        <v>181.2727272727273</v>
+        <v>179.6363636363636</v>
       </c>
       <c r="AR166" t="n">
         <v>74.90909090909091</v>
       </c>
       <c r="AS166" t="n">
-        <v>-0.04472253518218941</v>
+        <v>0.06290880668723749</v>
       </c>
       <c r="AT166" t="n">
         <v>23.5</v>
@@ -35017,16 +35017,16 @@
         <v>-0.2529848064417309</v>
       </c>
       <c r="AP167" t="n">
-        <v>24.55555555555556</v>
+        <v>24.4</v>
       </c>
       <c r="AQ167" t="n">
-        <v>183.8888888888889</v>
+        <v>182.5</v>
       </c>
       <c r="AR167" t="n">
-        <v>81.77777777777777</v>
+        <v>81.3</v>
       </c>
       <c r="AS167" t="n">
-        <v>2.413297296616348</v>
+        <v>2.228005128804551</v>
       </c>
       <c r="AT167" t="n">
         <v>26.55555555555556</v>
@@ -35650,16 +35650,16 @@
         <v>0.1384549246931496</v>
       </c>
       <c r="AT170" t="n">
-        <v>24.125</v>
+        <v>24.42857142857143</v>
       </c>
       <c r="AU170" t="n">
-        <v>184.125</v>
+        <v>185.1428571428571</v>
       </c>
       <c r="AV170" t="n">
-        <v>69.5</v>
+        <v>69</v>
       </c>
       <c r="AW170" t="n">
-        <v>-0.4087986748289246</v>
+        <v>-0.4245261640263082</v>
       </c>
       <c r="AX170" t="n">
         <v>24.71428571428572</v>
@@ -36661,16 +36661,16 @@
         </is>
       </c>
       <c r="AL175" t="n">
-        <v>26.72727272727273</v>
+        <v>27.18181818181818</v>
       </c>
       <c r="AM175" t="n">
-        <v>181.7272727272727</v>
+        <v>182.6363636363636</v>
       </c>
       <c r="AN175" t="n">
-        <v>77.27272727272727</v>
+        <v>77.45454545454545</v>
       </c>
       <c r="AO175" t="n">
-        <v>0.3825213889458405</v>
+        <v>0.3923657189948734</v>
       </c>
       <c r="AP175" t="n">
         <v>28.7</v>
@@ -37270,16 +37270,16 @@
         <v>0.07452511614509638</v>
       </c>
       <c r="AP178" t="n">
-        <v>25.72727272727273</v>
+        <v>26</v>
       </c>
       <c r="AQ178" t="n">
-        <v>182.5454545454545</v>
+        <v>183.6</v>
       </c>
       <c r="AR178" t="n">
-        <v>76.81818181818181</v>
+        <v>76.7</v>
       </c>
       <c r="AS178" t="n">
-        <v>0.3208302539719007</v>
+        <v>0.2607798406727997</v>
       </c>
       <c r="AT178" t="n">
         <v>25.11111111111111</v>
@@ -37662,16 +37662,16 @@
         </is>
       </c>
       <c r="AL180" t="n">
-        <v>24.90909090909091</v>
+        <v>24</v>
       </c>
       <c r="AM180" t="n">
-        <v>182.6363636363636</v>
+        <v>181</v>
       </c>
       <c r="AN180" t="n">
         <v>74.63636363636364</v>
       </c>
       <c r="AO180" t="n">
-        <v>-0.07753696867896591</v>
+        <v>0.03009437319046099</v>
       </c>
       <c r="AP180" t="n">
         <v>24.7</v>
@@ -37698,16 +37698,16 @@
         <v>-0.2449635004758522</v>
       </c>
       <c r="AX180" t="n">
-        <v>28.85714285714286</v>
+        <v>28.125</v>
       </c>
       <c r="AY180" t="n">
-        <v>184.8571428571429</v>
+        <v>183</v>
       </c>
       <c r="AZ180" t="n">
-        <v>78.28571428571429</v>
+        <v>78.125</v>
       </c>
       <c r="BA180" t="n">
-        <v>0.5606334461901296</v>
+        <v>0.5606012177286595</v>
       </c>
       <c r="BB180" t="n">
         <v>26.16666666666667</v>
@@ -38918,16 +38918,16 @@
         <v>2.090840796788025</v>
       </c>
       <c r="AT186" t="n">
-        <v>28.85714285714286</v>
+        <v>28.125</v>
       </c>
       <c r="AU186" t="n">
-        <v>184.8571428571429</v>
+        <v>183</v>
       </c>
       <c r="AV186" t="n">
-        <v>78.28571428571429</v>
+        <v>78.125</v>
       </c>
       <c r="AW186" t="n">
-        <v>0.5606334461901296</v>
+        <v>0.5606012177286596</v>
       </c>
       <c r="AX186" t="n">
         <v>26.42857142857143</v>
@@ -39310,16 +39310,16 @@
         <v>3.668230614978071</v>
       </c>
       <c r="AP188" t="n">
-        <v>25</v>
+        <v>24.09090909090909</v>
       </c>
       <c r="AQ188" t="n">
-        <v>183.0909090909091</v>
+        <v>181.4545454545455</v>
       </c>
       <c r="AR188" t="n">
         <v>74.45454545454545</v>
       </c>
       <c r="AS188" t="n">
-        <v>-0.1326652169535504</v>
+        <v>-0.0250338750841235</v>
       </c>
       <c r="AT188" t="n">
         <v>24.11111111111111</v>
@@ -39505,28 +39505,28 @@
         </is>
       </c>
       <c r="AL189" t="n">
-        <v>25.63636363636364</v>
+        <v>25.9</v>
       </c>
       <c r="AM189" t="n">
-        <v>183.0909090909091</v>
+        <v>184.2</v>
       </c>
       <c r="AN189" t="n">
-        <v>77.27272727272727</v>
+        <v>77.2</v>
       </c>
       <c r="AO189" t="n">
-        <v>0.4455251012596514</v>
+        <v>0.3979441726893255</v>
       </c>
       <c r="AP189" t="n">
-        <v>27.90909090909091</v>
+        <v>28.36363636363636</v>
       </c>
       <c r="AQ189" t="n">
-        <v>179.9090909090909</v>
+        <v>180.8181818181818</v>
       </c>
       <c r="AR189" t="n">
-        <v>76.81818181818181</v>
+        <v>77</v>
       </c>
       <c r="AS189" t="n">
-        <v>0.2840780884555111</v>
+        <v>0.293922418504544</v>
       </c>
       <c r="AT189" t="n">
         <v>25.5</v>
@@ -39921,16 +39921,16 @@
         <v>2.090840796788025</v>
       </c>
       <c r="AP191" t="n">
-        <v>26.63636363636364</v>
+        <v>27</v>
       </c>
       <c r="AQ191" t="n">
-        <v>182.0909090909091</v>
+        <v>183.1</v>
       </c>
       <c r="AR191" t="n">
-        <v>77.63636363636364</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AS191" t="n">
-        <v>0.458650874658362</v>
+        <v>0.4123825234279072</v>
       </c>
       <c r="AT191" t="n">
         <v>26.875</v>
@@ -40349,16 +40349,16 @@
         <v>-0.2605477520667023</v>
       </c>
       <c r="AX193" t="n">
-        <v>26.5</v>
+        <v>26.11111111111111</v>
       </c>
       <c r="AY193" t="n">
-        <v>182.875</v>
+        <v>181.4444444444445</v>
       </c>
       <c r="AZ193" t="n">
         <v>77</v>
       </c>
       <c r="BA193" t="n">
-        <v>0.6873879851518298</v>
+        <v>0.673275499968112</v>
       </c>
       <c r="BB193" t="inlineStr"/>
       <c r="BC193" t="inlineStr"/>
@@ -40717,16 +40717,16 @@
         </is>
       </c>
       <c r="AL195" t="n">
-        <v>25.18181818181818</v>
+        <v>24.27272727272727</v>
       </c>
       <c r="AM195" t="n">
-        <v>183.0909090909091</v>
+        <v>181.4545454545455</v>
       </c>
       <c r="AN195" t="n">
         <v>74.72727272727273</v>
       </c>
       <c r="AO195" t="n">
-        <v>-0.1208520208947109</v>
+        <v>-0.01322067902528396</v>
       </c>
       <c r="AP195" t="n">
         <v>28</v>
@@ -40914,16 +40914,16 @@
         </is>
       </c>
       <c r="AL196" t="n">
-        <v>28.09090909090909</v>
+        <v>28.54545454545455</v>
       </c>
       <c r="AM196" t="n">
-        <v>180.8181818181818</v>
+        <v>181.7272727272727</v>
       </c>
       <c r="AN196" t="n">
-        <v>77.09090909090909</v>
+        <v>77.27272727272727</v>
       </c>
       <c r="AO196" t="n">
-        <v>0.3293620066810626</v>
+        <v>0.3392063367300956</v>
       </c>
       <c r="AP196" t="n">
         <v>26.36363636363636</v>

</xml_diff>